<commit_message>
refactor: align run-single-lighthouse.ts with run-all-lighthouse config (#6)
- Refactor run-single-lighthouse.ts to match run-all-lighthouse configuration
- Update Excel template with latest changes
</commit_message>
<xml_diff>
--- a/template/CheQ_Website_Production_Lighthouse Report_Template_08222025_v2.2.xlsx
+++ b/template/CheQ_Website_Production_Lighthouse Report_Template_08222025_v2.2.xlsx
@@ -5,29 +5,29 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cheqteams-my.sharepoint.com/personal/vwlabajo_cheqsystems_com/Documents/Documents/Team - Performance Testing/PT - Documentation/CheQ Website Production Page Speed Insight/Template/Non macro/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VonWebsterDLabajo\VS Code\Private-Lighthouse-Automation\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1660" documentId="8_{92750536-FAD4-4F92-B76C-EB177816CE20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2021DC98-CD2A-4025-9681-07602F5954BD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CBF4F06-0752-4EB4-AE97-46A26D1E17C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A3D68101-3EA1-4AB8-9C35-12A619CAE77F}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="Formula_Sheet" sheetId="15" state="hidden" r:id="rId2"/>
-    <sheet name="01_Home" sheetId="7" r:id="rId3"/>
-    <sheet name="02_Testing" sheetId="8" r:id="rId4"/>
-    <sheet name="03_About" sheetId="9" r:id="rId5"/>
-    <sheet name="04_News" sheetId="10" r:id="rId6"/>
-    <sheet name="05_Careers" sheetId="11" r:id="rId7"/>
-    <sheet name="06_Contact" sheetId="12" r:id="rId8"/>
-    <sheet name="07_Privacy" sheetId="13" r:id="rId9"/>
-    <sheet name="08_Game Testing" sheetId="14" r:id="rId10"/>
+    <sheet name="01_Home" sheetId="7" r:id="rId2"/>
+    <sheet name="02_Testing" sheetId="8" r:id="rId3"/>
+    <sheet name="03_About" sheetId="9" r:id="rId4"/>
+    <sheet name="04_News" sheetId="10" r:id="rId5"/>
+    <sheet name="05_Careers" sheetId="11" r:id="rId6"/>
+    <sheet name="06_Contact" sheetId="12" r:id="rId7"/>
+    <sheet name="07_Privacy" sheetId="13" r:id="rId8"/>
+    <sheet name="08_Game Testing" sheetId="14" r:id="rId9"/>
+    <sheet name="Formula_Sheet" sheetId="15" state="hidden" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="cacheRange">Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!</definedName>
-    <definedName name="formulaPerformanceSheet" localSheetId="1">Formula_Sheet!$N$6:$N$35</definedName>
-    <definedName name="performanceRange" localSheetId="1">Summary!#REF!</definedName>
+    <definedName name="formulaPerformanceSheet" localSheetId="9">Formula_Sheet!$N$6:$N$35</definedName>
+    <definedName name="performanceRange" localSheetId="9">Summary!#REF!</definedName>
     <definedName name="performanceRange" localSheetId="0">Summary!#REF!</definedName>
     <definedName name="performanceValueRange" comment="This variable refers to the performance of all pages, for devices, cache, and without cache.">Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!,Summary!#REF!</definedName>
   </definedNames>
@@ -1013,7 +1013,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1255,27 +1255,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2526,182 +2533,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E531A025-BA5E-4614-A80F-6870F52C8D7D}">
-  <sheetPr codeName="Sheet9"/>
-  <dimension ref="B2:E27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="2.6640625" customWidth="1"/>
-    <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="95.109375" customWidth="1"/>
-    <col min="6" max="6" width="2.6640625" customWidth="1"/>
-    <col min="7" max="8" width="16.5546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C2" s="87">
-        <f>Summary!D34</f>
-        <v>0</v>
-      </c>
-      <c r="D2" s="88"/>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" s="89" t="str">
-        <f>Summary!B35</f>
-        <v>08_Game Testing</v>
-      </c>
-      <c r="C3" s="92" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="17"/>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="90"/>
-      <c r="C4" s="93"/>
-      <c r="D4" s="19" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" s="17"/>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B5" s="90"/>
-      <c r="C5" s="93" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="17"/>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="91"/>
-      <c r="C6" s="94"/>
-      <c r="D6" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="E6" s="17"/>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="E7" s="15"/>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" s="95">
-        <f>E5</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="96"/>
-      <c r="E9" s="97"/>
-    </row>
-    <row r="10" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="98"/>
-      <c r="D10" s="99"/>
-    </row>
-    <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" s="100"/>
-      <c r="D11" s="101"/>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B24" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B25" t="s">
-        <v>39</v>
-      </c>
-      <c r="C25" s="95">
-        <f>E5</f>
-        <v>0</v>
-      </c>
-      <c r="D25" s="96"/>
-      <c r="E25" s="97"/>
-    </row>
-    <row r="26" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" t="s">
-        <v>40</v>
-      </c>
-      <c r="C26" s="102"/>
-      <c r="D26" s="103"/>
-      <c r="E26" s="104"/>
-    </row>
-    <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" t="s">
-        <v>41</v>
-      </c>
-      <c r="C27" s="100"/>
-      <c r="D27" s="105"/>
-      <c r="E27" s="101"/>
-    </row>
-  </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C804090-FBAE-47C4-8581-16407B81F6C3}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="I3:AP64"/>
@@ -6592,7 +6423,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE5F55B9-0083-44F1-9B1A-CBDC42D16A9A}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="B1:E27"/>
@@ -6728,16 +6559,16 @@
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="102"/>
-      <c r="D26" s="103"/>
-      <c r="E26" s="104"/>
+      <c r="C26" s="98"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="99"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
       <c r="C27" s="100"/>
-      <c r="D27" s="105"/>
+      <c r="D27" s="103"/>
       <c r="E27" s="101"/>
     </row>
   </sheetData>
@@ -6757,7 +6588,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{411D02A4-EB3E-4DA1-B09D-21DE109734FA}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="B1:E30"/>
@@ -6845,6 +6676,7 @@
       </c>
       <c r="C10" s="98"/>
       <c r="D10" s="99"/>
+      <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
@@ -6852,6 +6684,7 @@
       </c>
       <c r="C11" s="100"/>
       <c r="D11" s="101"/>
+      <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C12" s="16"/>
@@ -6905,20 +6738,187 @@
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="102"/>
-      <c r="D26" s="103"/>
-      <c r="E26" s="104"/>
+      <c r="C26" s="98"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="99"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
       <c r="C27" s="100"/>
-      <c r="D27" s="105"/>
+      <c r="D27" s="103"/>
       <c r="E27" s="101"/>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C30" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C11:D11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE6E692C-8D28-41B6-9AD3-6D28106F46D8}">
+  <sheetPr codeName="Sheet4"/>
+  <dimension ref="B1:E27"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="2.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="95.5546875" customWidth="1"/>
+    <col min="6" max="6" width="2.6640625" customWidth="1"/>
+    <col min="7" max="8" width="16.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="87">
+        <f>Summary!D14</f>
+        <v>0</v>
+      </c>
+      <c r="D2" s="88"/>
+    </row>
+    <row r="3" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="89" t="str">
+        <f>Summary!B15</f>
+        <v>03_About</v>
+      </c>
+      <c r="C3" s="92" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="17"/>
+    </row>
+    <row r="4" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="90"/>
+      <c r="C4" s="93"/>
+      <c r="D4" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="17"/>
+    </row>
+    <row r="5" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="90"/>
+      <c r="C5" s="93" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="17"/>
+    </row>
+    <row r="6" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="91"/>
+      <c r="C6" s="94"/>
+      <c r="D6" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" s="17"/>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="E7" s="15"/>
+    </row>
+    <row r="8" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="95">
+        <f>E5</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="96"/>
+      <c r="E9" s="97"/>
+    </row>
+    <row r="10" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="98"/>
+      <c r="D10" s="99"/>
+      <c r="E10" s="23"/>
+    </row>
+    <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="100"/>
+      <c r="D11" s="101"/>
+      <c r="E11" s="23"/>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+    </row>
+    <row r="24" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B24" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" s="95">
+        <f>E5</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="96"/>
+      <c r="E25" s="97"/>
+    </row>
+    <row r="26" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B26" t="s">
+        <v>40</v>
+      </c>
+      <c r="C26" s="98"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="99"/>
+    </row>
+    <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B27" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="100"/>
+      <c r="D27" s="103"/>
+      <c r="E27" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -6938,8 +6938,8 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE6E692C-8D28-41B6-9AD3-6D28106F46D8}">
-  <sheetPr codeName="Sheet4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{818F93A7-7B41-43F7-893B-45F15C78D9DC}">
+  <sheetPr codeName="Sheet5"/>
   <dimension ref="B1:E27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -6954,15 +6954,15 @@
     <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C2" s="87">
-        <f>Summary!D14</f>
+        <f>Summary!D18</f>
         <v>0</v>
       </c>
       <c r="D2" s="88"/>
     </row>
     <row r="3" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="89" t="str">
-        <f>Summary!B15</f>
-        <v>03_About</v>
+        <f>Summary!B19</f>
+        <v>04_News</v>
       </c>
       <c r="C3" s="92" t="s">
         <v>13</v>
@@ -7025,6 +7025,7 @@
       </c>
       <c r="C10" s="98"/>
       <c r="D10" s="99"/>
+      <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
@@ -7032,6 +7033,7 @@
       </c>
       <c r="C11" s="100"/>
       <c r="D11" s="101"/>
+      <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C12" s="16"/>
@@ -7053,6 +7055,18 @@
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
     </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+    </row>
     <row r="24" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>42</v>
@@ -7073,16 +7087,16 @@
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="102"/>
-      <c r="D26" s="103"/>
-      <c r="E26" s="104"/>
+      <c r="C26" s="98"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="99"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
       <c r="C27" s="100"/>
-      <c r="D27" s="105"/>
+      <c r="D27" s="103"/>
       <c r="E27" s="101"/>
     </row>
   </sheetData>
@@ -7103,9 +7117,9 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{818F93A7-7B41-43F7-893B-45F15C78D9DC}">
-  <sheetPr codeName="Sheet5"/>
-  <dimension ref="B1:E27"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F8CF2DB-0020-469F-8BA3-7660EE65C4AC}">
+  <sheetPr codeName="Sheet6"/>
+  <dimension ref="B1:E29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
@@ -7113,21 +7127,21 @@
     <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="95.5546875" customWidth="1"/>
     <col min="6" max="6" width="2.6640625" customWidth="1"/>
-    <col min="7" max="8" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C2" s="87">
-        <f>Summary!D18</f>
+        <f>Summary!D22</f>
         <v>0</v>
       </c>
       <c r="D2" s="88"/>
     </row>
     <row r="3" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="89" t="str">
-        <f>Summary!B19</f>
-        <v>04_News</v>
+        <f>Summary!B23</f>
+        <v>05_Careers</v>
       </c>
       <c r="C3" s="92" t="s">
         <v>13</v>
@@ -7190,6 +7204,7 @@
       </c>
       <c r="C10" s="98"/>
       <c r="D10" s="99"/>
+      <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
@@ -7197,6 +7212,7 @@
       </c>
       <c r="C11" s="100"/>
       <c r="D11" s="101"/>
+      <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C12" s="16"/>
@@ -7250,17 +7266,20 @@
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="102"/>
-      <c r="D26" s="103"/>
-      <c r="E26" s="104"/>
+      <c r="C26" s="98"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="99"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
       <c r="C27" s="100"/>
-      <c r="D27" s="105"/>
+      <c r="D27" s="103"/>
       <c r="E27" s="101"/>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C29" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -7280,9 +7299,9 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F8CF2DB-0020-469F-8BA3-7660EE65C4AC}">
-  <sheetPr codeName="Sheet6"/>
-  <dimension ref="B1:E29"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7736922B-F394-4ACF-802A-EAB14293D18C}">
+  <sheetPr codeName="Sheet7"/>
+  <dimension ref="B1:E27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
@@ -7290,21 +7309,21 @@
     <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="95.5546875" customWidth="1"/>
     <col min="6" max="6" width="2.6640625" customWidth="1"/>
-    <col min="7" max="7" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="16.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C2" s="87">
-        <f>Summary!D22</f>
+        <f>Summary!D26</f>
         <v>0</v>
       </c>
       <c r="D2" s="88"/>
     </row>
     <row r="3" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="89" t="str">
-        <f>Summary!B23</f>
-        <v>05_Careers</v>
+        <f>Summary!B27</f>
+        <v>06_Contact</v>
       </c>
       <c r="C3" s="92" t="s">
         <v>13</v>
@@ -7359,7 +7378,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="96"/>
-      <c r="E9" s="97"/>
+      <c r="E9" s="104"/>
     </row>
     <row r="10" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
@@ -7427,20 +7446,17 @@
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="102"/>
-      <c r="D26" s="103"/>
-      <c r="E26" s="104"/>
+      <c r="C26" s="98"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="99"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
       <c r="C27" s="100"/>
-      <c r="D27" s="105"/>
+      <c r="D27" s="103"/>
       <c r="E27" s="101"/>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C29" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -7460,9 +7476,9 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7736922B-F394-4ACF-802A-EAB14293D18C}">
-  <sheetPr codeName="Sheet7"/>
-  <dimension ref="B1:E27"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1D6D5E4-BFAB-41B7-A265-68420CAFEDDE}">
+  <sheetPr codeName="Sheet8"/>
+  <dimension ref="B2:E27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
@@ -7473,18 +7489,17 @@
     <col min="7" max="8" width="16.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C2" s="87">
-        <f>Summary!D26</f>
+        <f>Summary!D30</f>
         <v>0</v>
       </c>
       <c r="D2" s="88"/>
     </row>
-    <row r="3" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" s="89" t="str">
-        <f>Summary!B27</f>
-        <v>06_Contact</v>
+        <f>Summary!B31</f>
+        <v>07_Privacy</v>
       </c>
       <c r="C3" s="92" t="s">
         <v>13</v>
@@ -7492,17 +7507,17 @@
       <c r="D3" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="17"/>
-    </row>
-    <row r="4" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E3" s="33"/>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4" s="90"/>
       <c r="C4" s="93"/>
       <c r="D4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="17"/>
-    </row>
-    <row r="5" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E4" s="35"/>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B5" s="90"/>
       <c r="C5" s="93" t="s">
         <v>15</v>
@@ -7510,15 +7525,15 @@
       <c r="D5" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="17"/>
-    </row>
-    <row r="6" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E5" s="36"/>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="91"/>
       <c r="C6" s="94"/>
       <c r="D6" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="17"/>
+      <c r="E6" s="34"/>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="14"/>
@@ -7547,6 +7562,7 @@
       </c>
       <c r="C10" s="98"/>
       <c r="D10" s="99"/>
+      <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
@@ -7554,6 +7570,7 @@
       </c>
       <c r="C11" s="100"/>
       <c r="D11" s="101"/>
+      <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C12" s="16"/>
@@ -7575,18 +7592,6 @@
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-    </row>
     <row r="24" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>42</v>
@@ -7607,16 +7612,16 @@
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="102"/>
-      <c r="D26" s="103"/>
-      <c r="E26" s="104"/>
+      <c r="C26" s="98"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="99"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
       <c r="C27" s="100"/>
-      <c r="D27" s="105"/>
+      <c r="D27" s="103"/>
       <c r="E27" s="101"/>
     </row>
   </sheetData>
@@ -7637,30 +7642,30 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1D6D5E4-BFAB-41B7-A265-68420CAFEDDE}">
-  <sheetPr codeName="Sheet8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E531A025-BA5E-4614-A80F-6870F52C8D7D}">
+  <sheetPr codeName="Sheet9"/>
   <dimension ref="B2:E27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
     <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="95.5546875" customWidth="1"/>
+    <col min="5" max="5" width="95.109375" customWidth="1"/>
     <col min="6" max="6" width="2.6640625" customWidth="1"/>
     <col min="7" max="8" width="16.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C2" s="87">
-        <f>Summary!D30</f>
+        <f>Summary!D34</f>
         <v>0</v>
       </c>
       <c r="D2" s="88"/>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" s="89" t="str">
-        <f>Summary!B31</f>
-        <v>07_Privacy</v>
+        <f>Summary!B35</f>
+        <v>08_Game Testing</v>
       </c>
       <c r="C3" s="92" t="s">
         <v>13</v>
@@ -7668,7 +7673,7 @@
       <c r="D3" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="33"/>
+      <c r="E3" s="17"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4" s="90"/>
@@ -7676,7 +7681,7 @@
       <c r="D4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="35"/>
+      <c r="E4" s="17"/>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B5" s="90"/>
@@ -7686,7 +7691,7 @@
       <c r="D5" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="36"/>
+      <c r="E5" s="17"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="91"/>
@@ -7694,19 +7699,19 @@
       <c r="D6" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="34"/>
+      <c r="E6" s="17"/>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="14"/>
       <c r="C7" s="14"/>
       <c r="E7" s="15"/>
     </row>
-    <row r="8" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>39</v>
       </c>
@@ -7723,6 +7728,7 @@
       </c>
       <c r="C10" s="98"/>
       <c r="D10" s="99"/>
+      <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
@@ -7730,6 +7736,7 @@
       </c>
       <c r="C11" s="100"/>
       <c r="D11" s="101"/>
+      <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C12" s="16"/>
@@ -7751,12 +7758,24 @@
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
     </row>
-    <row r="24" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>39</v>
       </c>
@@ -7771,16 +7790,16 @@
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="102"/>
-      <c r="D26" s="103"/>
-      <c r="E26" s="104"/>
+      <c r="C26" s="98"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="99"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
       <c r="C27" s="100"/>
-      <c r="D27" s="105"/>
+      <c r="D27" s="103"/>
       <c r="E27" s="101"/>
     </row>
   </sheetData>

</xml_diff>